<commit_message>
refactor(ui): atualiza comportamento de bottom sheets e filtro do mapa
- fix: expande bottom sheets automaticamente, corrigindo labels e alinhamento de ícones
- refactor: altera filtro do mapa para toggle individual por PointType via Map<PointType, Boolean>
</commit_message>
<xml_diff>
--- a/scripts/dados/sao_goncalo_ecopontos_rio_v2.xlsx
+++ b/scripts/dados/sao_goncalo_ecopontos_rio_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\temp\projeto-tcc\4-Documentos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\temp\projeto-tcc\automatic-happiness\scripts\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C281114-135D-43F1-932A-201591FA4E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50228C63-1FDC-4FB0-8910-C2B5F9BA3BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15585" yWindow="30" windowWidth="13215" windowHeight="14685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
   <si>
     <t>IDENTIDADE</t>
   </si>
@@ -185,7 +185,10 @@
     <t>benefits_program</t>
   </si>
   <si>
-    <t>Dinheiro digital creditado em cartão para uso em conta corrente ou estabelecimentos de São Gonçalo</t>
+    <t>Dinheiro digital creditado em cartão (uso em conta corrente ou estabelecimentos de São Gonçalo)</t>
+  </si>
+  <si>
+    <t>Programa Limpa São Gonçalo</t>
   </si>
 </sst>
 </file>
@@ -751,7 +754,7 @@
     <col min="15" max="15" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.42578125" customWidth="1"/>
+    <col min="18" max="18" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="87.7109375" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -899,7 +902,9 @@
       </c>
       <c r="P3" s="13"/>
       <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
+      <c r="R3" s="13" t="s">
+        <v>50</v>
+      </c>
       <c r="S3" s="13" t="s">
         <v>49</v>
       </c>
@@ -954,7 +959,9 @@
       </c>
       <c r="P4" s="16"/>
       <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
+      <c r="R4" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="S4" s="16" t="s">
         <v>49</v>
       </c>
@@ -1008,7 +1015,9 @@
       </c>
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
-      <c r="R5" s="13"/>
+      <c r="R5" s="13" t="s">
+        <v>50</v>
+      </c>
       <c r="S5" s="13" t="s">
         <v>49</v>
       </c>

</xml_diff>